<commit_message>
updated FCM algorithm (faster) and reclustering
</commit_message>
<xml_diff>
--- a/clustering/cluster_validation.xlsx
+++ b/clustering/cluster_validation.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,100 +459,66 @@
       <c r="A2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="B2" t="n">
-        <v>0</v>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
       </c>
       <c r="C2" t="n">
-        <v>0.05327941125230271</v>
+        <v>0.3602856351660009</v>
       </c>
       <c r="D2" t="n">
-        <v>0.7100318774882641</v>
+        <v>0.8041139883661723</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9438175270108043</v>
+        <v>0.9033853541416567</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9384814103585983</v>
+        <v>0.9016554207363513</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="n">
-        <v>1</v>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SU</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>0.09165709121972587</v>
+        <v>0.1442876346072846</v>
       </c>
       <c r="D3" t="n">
-        <v>0.4500485013962341</v>
+        <v>0.9546115187804232</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9519807923169267</v>
+        <v>0.9375750300120047</v>
       </c>
       <c r="F3" t="n">
-        <v>0.95575727315251</v>
+        <v>0.9783441716158835</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="n">
-        <v>2</v>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DSU</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>0.09653073994658849</v>
+        <v>0.2111387106473778</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7998734783190444</v>
+        <v>0.9366560281188716</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9538055222088836</v>
+        <v>0.9357503001200479</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9683529590596233</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.09183355276061106</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.8827560012203413</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.9598559423769507</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.9758154712178962</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.09861037359932748</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.8632341167734748</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.8553661464585834</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.963177652307022</v>
+        <v>0.9721729865840283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
addded  cluster selection file
</commit_message>
<xml_diff>
--- a/clustering/cluster_validation.xlsx
+++ b/clustering/cluster_validation.xlsx
@@ -465,16 +465,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.3602856351660009</v>
+        <v>0.3664487834283238</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8041139883661723</v>
+        <v>0.7969364371082429</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9033853541416567</v>
+        <v>0.9015606242496997</v>
       </c>
       <c r="F2" t="n">
-        <v>0.9016554207363513</v>
+        <v>0.8990421332062494</v>
       </c>
     </row>
     <row r="3">
@@ -487,16 +487,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.1442876346072846</v>
+        <v>0.142867414848957</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9546115187804232</v>
+        <v>0.9555487778975927</v>
       </c>
       <c r="E3" t="n">
-        <v>0.9375750300120047</v>
+        <v>0.946986794717887</v>
       </c>
       <c r="F3" t="n">
-        <v>0.9783441716158835</v>
+        <v>0.9790190699252201</v>
       </c>
     </row>
     <row r="4">
@@ -509,16 +509,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.2111387106473778</v>
+        <v>0.2164525854339497</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9366560281188716</v>
+        <v>0.9335398033621432</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9357503001200479</v>
+        <v>0.9337334933973589</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9721729865840283</v>
+        <v>0.9716833473958796</v>
       </c>
     </row>
   </sheetData>

</xml_diff>